<commit_message>
GJP发票导出: hide the GL lookup sheet in the exported workbook
GL is a VLOOKUP helper table, not data. Hiding it (sheet_state=hidden)
keeps the G/L column formula working while the export looks like a
single 电子发票 tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/src/assets/gjp_invoice_template.xlsx
+++ b/backend/src/assets/gjp_invoice_template.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="11925" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="11925" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="电子发票" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="GL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="GL" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
GJP发票导出: add 电子客票号码 to column U; open workbook at top-left
- write ticket number into column U (new 电子客票号码 header), kept as text
  so leading zeros survive
- reset the sheet view (topLeftCell/selection -> A1) so the exported file
  opens at the top instead of scrolled to the old data's last rows
- show 客票号 in the preview table

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/src/assets/gjp_invoice_template.xlsx
+++ b/backend/src/assets/gjp_invoice_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="11925" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="11925" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="电子发票" sheetId="1" state="visible" r:id="rId1"/>
@@ -3126,7 +3126,11 @@
           <t>发票号</t>
         </is>
       </c>
-      <c r="U7" s="253" t="n"/>
+      <c r="U7" s="252" t="inlineStr">
+        <is>
+          <t>电子客票号码</t>
+        </is>
+      </c>
       <c r="V7" s="253" t="n"/>
       <c r="W7" s="254" t="inlineStr">
         <is>

</xml_diff>